<commit_message>
chore: sincronizacion completa del backend
Incluye todos los cambios pendientes:
- Servicios, ETLs, handlers de orquestador
- Scripts de monitoreo y predicciones
- Tests actualizados
- Configuraciones de infraestructura
- Nuevos endpoints API y rutas
- Tareas Celery (anomaly_tasks, etl_tasks, push_tasks)
- Integracion whatsapp_bot y notificaciones
- Documentacion y configuraciones
</commit_message>
<xml_diff>
--- a/data/onedrive/Comunidades_Energeticas_Avance.xlsx
+++ b/data/onedrive/Comunidades_Energeticas_Avance.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29930"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -3906,12 +3906,11 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="8f154a8c-a0d7-469f-a565-81a8dee811c9" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4103,15 +4102,16 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="8f154a8c-a0d7-469f-a565-81a8dee811c9" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0787518D-69BD-4E45-AC35-D1E5AC391598}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51E095F6-BF66-41A9-AB03-40D964033B2A}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4119,5 +4119,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51E095F6-BF66-41A9-AB03-40D964033B2A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0787518D-69BD-4E45-AC35-D1E5AC391598}"/>
 </file>
</xml_diff>